<commit_message>
feat: Dissolve/DissolveRev 할 때 보여줄 파티클 이펙트 추가
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/PreLoadAssetData.xlsx
+++ b/JsonConverter/ExcelFiles/PreLoadAssetData.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="64">
   <si>
     <t>아이디
 는 상관 없음</t>
@@ -211,6 +211,18 @@
   </si>
   <si>
     <t>buff_fire_force</t>
+  </si>
+  <si>
+    <t>Dissolve</t>
+  </si>
+  <si>
+    <t>Particle/Dissolve</t>
+  </si>
+  <si>
+    <t>DissolveRev</t>
+  </si>
+  <si>
+    <t>Particle/DissolveRev</t>
   </si>
 </sst>
 </file>
@@ -1022,6 +1034,28 @@
         <v>9</v>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>